<commit_message>
scan: seg6 2026-09-28 15:54 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq7_2026-09-24.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>68.66754017944093</v>
+        <v>68.66754019650855</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>26.83106226527447</v>
+        <v>26.83106218996431</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.685524105208017</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.957899931676202</v>
+        <v>1.957899931099302</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>71.16375653384426</v>
+        <v>71.16375683481112</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>21.74317861808185</v>
+        <v>21.7431787825884</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.661943371713502</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.1545851921015624</v>
+        <v>0.1545851918439826</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>58.27249352056474</v>
+        <v>58.27249355224106</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>7.932196192235401</v>
+        <v>7.932196171050655</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>8.584258392238151</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.2035670185563913</v>
+        <v>0.2035670185769997</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>65.27530100844888</v>
+        <v>65.27530100318893</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>17.43169738044881</v>
+        <v>17.43169736750527</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>4.346659824971685</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>2.804177271951342</v>
+        <v>2.804177272157419</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>61.79438096910025</v>
+        <v>61.79438103867085</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>22.30944713874011</v>
+        <v>22.3094471552436</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>3.17558471647802</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>1.427628113530257</v>
+        <v>1.427628112087846</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>64.70178542243417</v>
+        <v>64.70178542397032</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>30.19848264230172</v>
+        <v>30.19848254674888</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.97728597061346</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.838392146505621</v>
+        <v>1.838392146546833</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>82.46147629892604</v>
+        <v>82.4614763644873</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>26.41998847336289</v>
+        <v>26.41998847705492</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>3.207844850229248</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>22.12763056599123</v>
+        <v>22.12763056310636</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>68.75851757113217</v>
+        <v>68.75851760375002</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>23.0177766446669</v>
+        <v>23.01777665367185</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>4.296995099878581</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>10.01171512616245</v>
+        <v>10.01171512533824</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>56.2409610598974</v>
+        <v>56.24096104817474</v>
       </c>
       <c r="I10" s="2" t="n">
         <v>10.98468357032213</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.2404680381680002</v>
+        <v>0.2404680369317802</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>60.50713019247176</v>
+        <v>60.50713018306762</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>37.9593694957364</v>
+        <v>37.95936948238987</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.650772025543959</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.2572289233710529</v>
+        <v>-0.257228923350441</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>63.31977508796878</v>
+        <v>63.31977517961854</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>45.20069356908386</v>
+        <v>45.20069381244598</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.4302284329160745</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.2442435278225092</v>
+        <v>0.2442435272146399</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>848.6490266520968</v>
+        <v>848.6490266520972</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>667</v>
@@ -1135,7 +1135,7 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>58.35151311088111</v>
+        <v>58.35151317067923</v>
       </c>
       <c r="I13" s="2" t="n">
         <v>16.3956978809125</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>7.923448355375294</v>
+        <v>7.9234483538298</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.54223832847885</v>
+        <v>60.54223831820774</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>28.12260908527933</v>
+        <v>28.12260914673256</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.4464859771818252</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>1.571134810165413</v>
+        <v>1.571134811813875</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>65.61060064347791</v>
+        <v>65.61060064388079</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>32.15373258712496</v>
+        <v>32.15373259400138</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.6827230607894571</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>26.13903972025008</v>
+        <v>26.13903972292927</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1297,7 +1297,7 @@
         <v>59.67954326340881</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>31.81749372299765</v>
+        <v>31.81749372378981</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.6040651995779337</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.0411138573501457</v>
+        <v>0.0411138574531673</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>62.55096456392263</v>
+        <v>62.55096454979986</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>44.75207660258552</v>
+        <v>44.75207661328924</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.4966982704420574</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.4467829363246536</v>
+        <v>0.4467829364482902</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>67.16033985741622</v>
+        <v>67.16033985970495</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>62.49451581861285</v>
+        <v>62.49451583781153</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.149941419890234</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2.941039513522171</v>
+        <v>2.941039513748819</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>741.7553124543479</v>
+        <v>741.7553124543483</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>261.5</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>65.14607024283248</v>
+        <v>65.14607035151424</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>37.45305621401626</v>
+        <v>37.45305625220068</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.5241372274217474</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>2.498773223236983</v>
+        <v>2.498773222618782</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1509,7 +1509,7 @@
         <v>56.57339564812207</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>21.00564399643293</v>
+        <v>21.00564400756689</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.5684408896010303</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>14.32666916373711</v>
+        <v>14.32666916301569</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>54.79130149746421</v>
+        <v>54.79130147505931</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>30.71886406188479</v>
+        <v>30.71886418578853</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.7554779489056903</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.482179917429894</v>
+        <v>1.482179918975275</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>72.06436265202319</v>
+        <v>72.06436274263918</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>30.0873080931078</v>
+        <v>30.08730806053153</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.8183871815292657</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.2901901870463977</v>
+        <v>0.2901901869433685</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>52.31573296216632</v>
+        <v>52.31573324599304</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>7.777975251298856</v>
+        <v>7.777975798880761</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.521466971058252</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.0785537194318382</v>
+        <v>0.07855370498717219</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>679.5983977201182</v>
+        <v>679.5983977201183</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>143</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>55.35700629578485</v>
+        <v>55.35700630691913</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>43.08147165708341</v>
+        <v>43.08147161332783</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.3510109837704807</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.84995822661089</v>
+        <v>0.8499582277029791</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>25.59756295088425</v>
+        <v>25.59756300519639</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>45.21174382248633</v>
+        <v>45.21174388568553</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.8078270744650331</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>17.01331216400285</v>
+        <v>17.01331214545746</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1810,7 +1810,7 @@
         <v/>
       </c>
       <c r="D26" s="2" t="n">
-        <v>654.7335124447823</v>
+        <v>654.7335124447824</v>
       </c>
       <c r="E26" s="2" t="n">
         <v>70.09999999999999</v>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>62.5563277255137</v>
+        <v>62.55632771123713</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>23.88546743705131</v>
+        <v>23.88546752293477</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1.165428532065079</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.329744655676096</v>
+        <v>1.329744655861554</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>67.5747872315535</v>
+        <v>67.57478715438286</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>40.2453612735793</v>
+        <v>40.2453613602517</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.972543201921374</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>1.135904390945412</v>
+        <v>1.135904391213288</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>51.16607913777997</v>
+        <v>51.16607896205471</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>23.07965734861008</v>
+        <v>23.07965741739384</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.6587897239350179</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-0.6874192295358634</v>
+        <v>-0.6874192281964873</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>604.2253956784632</v>
+        <v>604.2253956784633</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>358.5</v>
@@ -1983,7 +1983,7 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>56.58499929025162</v>
+        <v>56.5849993229416</v>
       </c>
       <c r="I29" s="2" t="n">
         <v>10.2918834106784</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>1.205389719781597</v>
+        <v>1.205389719060376</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>52.09765773867952</v>
+        <v>52.09765784986006</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>23.18118075614707</v>
+        <v>23.18118076870248</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.3336766004557814</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-0.9119035863905848</v>
+        <v>-0.9119035856693758</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>47.39828994768262</v>
+        <v>47.39828998574609</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>27.40172096882054</v>
+        <v>27.40172094996863</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.392094524945494</v>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>51.68650898588238</v>
+        <v>51.68650901865525</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>33.13407064711544</v>
+        <v>33.13407067885349</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.9088189620361444</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-14.34582857106119</v>
+        <v>-14.34582857827348</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>55.88810673368297</v>
+        <v>55.88810671340467</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>21.93956159438618</v>
+        <v>21.93956159338195</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>1.663121215559225</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.3309913462336702</v>
+        <v>0.3309913466457752</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>567.5678250447919</v>
+        <v>567.567825044792</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>179</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.78139645688736</v>
+        <v>57.78139645137507</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>16.64239963502372</v>
+        <v>16.6423997007581</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.409581288192835</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.5771740225456057</v>
+        <v>0.577174022834082</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>58.52992311042029</v>
+        <v>58.52992308126178</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>31.80823292065671</v>
+        <v>31.80823287534841</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.3625300479778954</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.7153760597761734</v>
+        <v>0.7153760601882788</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>532.8771635878553</v>
+        <v>532.8771635878538</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>42</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>55.36330491003964</v>
+        <v>55.36330474930742</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>21.72365912656409</v>
+        <v>21.72365924050072</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.304760356772791</v>
@@ -2407,7 +2407,7 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>31.69502272070223</v>
+        <v>31.69503153248954</v>
       </c>
       <c r="I37" s="2" t="n">
         <v>32.59321928795873</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.4112821273959026</v>
+        <v>0.4112821095165779</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>55.78584459711723</v>
+        <v>55.785844708163</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>9.63034803165497</v>
+        <v>9.630348031654968</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.4155415414568079</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>0.0285085087610165</v>
+        <v>0.0285085086476898</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>52.60058349474705</v>
+        <v>52.60058351316243</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>8.975604866372624</v>
+        <v>8.975604874723546</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.7337314238331761</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.0452549455209726</v>
+        <v>0.0452549454591612</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         <v>0</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>54.03842995857126</v>
+        <v>54.03842997062653</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>25.32562450535045</v>
+        <v>25.32562451096538</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.2435764880321545</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.5147660984740838</v>
+        <v>-0.5147660984946953</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>503.5177132338883</v>
+        <v>503.5177132338882</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>540</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>52.96310896554198</v>
+        <v>52.96310899466217</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>27.72772532795458</v>
+        <v>27.72772531839418</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.4416483554075971</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-7.160934444678468</v>
+        <v>-7.160934445296718</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>48.37480315689982</v>
+        <v>48.37480316821787</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>13.99015890311896</v>
+        <v>13.99015890846122</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.4652378730945042</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>61.13659917622377</v>
+        <v>61.13659915155117</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>19.10493702824942</v>
+        <v>19.10493708206357</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>1.136273133488234</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>1.105702871024606</v>
+        <v>1.105702871333707</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>47.36817235395961</v>
+        <v>47.36817246581801</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>25.3372896519572</v>
+        <v>25.33728966958646</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.4657350026052051</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.0040183609673321</v>
+        <v>-0.0040183611321781</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>455.8431542223493</v>
+        <v>455.8431542223494</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>51.4</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>55.49458298889965</v>
+        <v>55.49458303328909</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>18.34498681348361</v>
+        <v>18.3449867841258</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>1.207504683192515</v>
@@ -2923,7 +2923,7 @@
         <v/>
       </c>
       <c r="D47" s="2" t="n">
-        <v>453.6553063381715</v>
+        <v>453.6553063381713</v>
       </c>
       <c r="E47" s="2" t="n">
         <v>1010</v>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>42.24014343378963</v>
+        <v>42.24014344628299</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>21.6727572603239</v>
+        <v>21.67275727779379</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.5335609419929919</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-23.92442062929137</v>
+        <v>-23.92442063197018</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>54.82247203367415</v>
+        <v>54.8224720189723</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>46.55901901780671</v>
+        <v>46.55901904509773</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.1434060592326219</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.1279232031810835</v>
+        <v>-0.1279232031604884</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>52.12765401353386</v>
+        <v>52.12765402325228</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>8.45661971303155</v>
+        <v>8.456619753008512</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>1.324830518212111</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.0971265221113212</v>
+        <v>0.0971265220804132</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,7 +3096,7 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>50.43995562705216</v>
+        <v>50.43995570404039</v>
       </c>
       <c r="I50" s="2" t="n">
         <v>22.54481023784425</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.09152553686680021</v>
+        <v>-0.0915255370728533</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>45.13497127902576</v>
+        <v>45.13497129517609</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>13.5093765477186</v>
+        <v>13.50937649122115</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.647273987081031</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0385486184269446</v>
+        <v>0.0385486183857277</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>418.694356960769</v>
+        <v>418.6943569607691</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>948</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>49.47095738651421</v>
+        <v>49.47095741242141</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.4440116737198</v>
+        <v>8.444011691681018</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.93264437588126</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>4.940413011726886</v>
+        <v>4.940413010902663</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>418.2524790326089</v>
+        <v>418.2524790326087</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>465.5</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>53.86008531524513</v>
+        <v>53.86008532407225</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>12.19947714076998</v>
+        <v>12.19947711498095</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5959109105149348</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>1.747680153761688</v>
+        <v>1.747680153452647</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3308,7 +3308,7 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>53.4041245814857</v>
+        <v>53.40412464597301</v>
       </c>
       <c r="I54" s="2" t="n">
         <v>19.310935800471</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.9186962191186684</v>
+        <v>0.9186962190156338</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>409.3218640015365</v>
+        <v>409.3218640015364</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>90.5</v>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>44.72886928218384</v>
+        <v>44.72886892065956</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>10.18479475023668</v>
+        <v>10.1847946646186</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>1.505333590988018</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.0176562700635355</v>
+        <v>0.0176562705992771</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>404.8845594177959</v>
+        <v>404.8845594177957</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>24.5</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>49.60827130951143</v>
+        <v>49.60827128143913</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>26.15023113565296</v>
+        <v>26.15023116888705</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.8650145154211294</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.1837762695736999</v>
+        <v>0.1837762696252162</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>402.7111623172824</v>
+        <v>402.7111623172892</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>44.2</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>55.11978925775367</v>
+        <v>55.11978952310063</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.06923076050597</v>
+        <v>29.06923083260857</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.40320428304767</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.4088516817993811</v>
+        <v>0.4088516819230153</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>402.3567160515234</v>
+        <v>402.3567160515287</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1110</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>50.70385318696061</v>
+        <v>50.70385319998633</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>11.1859026832861</v>
+        <v>11.18590270123124</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.4290261573668845</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-10.52299224449052</v>
+        <v>-10.5229922432542</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>50.32722816369422</v>
+        <v>50.32722816895669</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>8.989604531200957</v>
+        <v>8.989604692640697</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>3.203068149522319</v>
@@ -3612,7 +3612,7 @@
         <v/>
       </c>
       <c r="D60" s="2" t="n">
-        <v>390.9473456525848</v>
+        <v>390.9473456525847</v>
       </c>
       <c r="E60" s="2" t="n">
         <v>505</v>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>54.97217804293678</v>
+        <v>54.97217806375415</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>17.02854771119858</v>
+        <v>17.02854771431543</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.03301322482184</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-6.705685453361482</v>
+        <v>-6.705685453196642</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>382.4710173027302</v>
+        <v>382.4710173027301</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>32.8</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>50.17423570190032</v>
+        <v>50.1742358134637</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>23.3015038919845</v>
+        <v>23.30150391297365</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.323416615282644</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.08838544489624869</v>
+        <v>-0.0883854448550398</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>378.2401478543657</v>
+        <v>378.2401478543658</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>46.65</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>34.9631523112588</v>
+        <v>34.96315223405169</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>31.58515629545469</v>
+        <v>31.58515635258613</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.3319491119899236</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.0625534502520366</v>
+        <v>-0.0625534501077995</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>48.1540629908425</v>
+        <v>48.15406298716601</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.04032663879525</v>
+        <v>23.04032668827005</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.2955256328703418</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-2.332987316064712</v>
+        <v>-2.332987316002886</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>45.92691714908729</v>
+        <v>45.9269171851949</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>16.5213547050591</v>
+        <v>16.52135472293203</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.5972748766961367</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.0746118402565468</v>
+        <v>-0.0746118402771541</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>369.59977602131</v>
+        <v>369.5997760213101</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>97.5</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>49.02842206738176</v>
+        <v>49.0284220944752</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>9.539050290251224</v>
+        <v>9.539050306776504</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.6590440111141078</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.0245580214517339</v>
+        <v>-0.0245580212044544</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>43.52159338725793</v>
+        <v>43.52159340238235</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>11.41364098983295</v>
+        <v>11.4136409625665</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.3222677259872201</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.1885271152800627</v>
+        <v>-0.1885271147649017</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>40.46448124114259</v>
+        <v>40.46448163914612</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>12.83135022062205</v>
+        <v>12.83135036525853</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>1.806491484531917</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.2613456656219943</v>
+        <v>-0.2613456663638074</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,7 +4050,7 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>57.25589860242721</v>
+        <v>57.2558986250877</v>
       </c>
       <c r="I68" s="2" t="n">
         <v>19.98805306399838</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>1.217486811571745</v>
+        <v>1.217486811777785</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>348.3542541384185</v>
+        <v>348.3542541384186</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>71.3</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>46.92396404749105</v>
+        <v>46.92396406438479</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>13.88576406815744</v>
+        <v>13.88576413953373</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.5174383721506689</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.0444866843022589</v>
+        <v>0.044486684353754</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>46.2396748846228</v>
+        <v>46.2396751519973</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>25.60654188612326</v>
+        <v>25.60654187287011</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.5507151254854856</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.2183728888659257</v>
+        <v>0.2183728885774385</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>57.41756280424846</v>
+        <v>57.41756283461797</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>19.91919288923067</v>
+        <v>19.91919289890828</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6419259175666775</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.5351916854060741</v>
+        <v>0.5351916854884915</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>44.69811226918988</v>
+        <v>44.69811224540418</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>13.70076766481684</v>
+        <v>13.70076773373744</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.366188600864838</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-3.595449209951754</v>
+        <v>-3.595449208921471</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>53.39391182458387</v>
+        <v>53.39391177200346</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15.04376319296496</v>
+        <v>15.04376320296989</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.7440767050085816</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.1865894953279119</v>
+        <v>0.186589495420639</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4354,7 +4354,7 @@
         <v/>
       </c>
       <c r="D74" s="2" t="n">
-        <v>336.4885879134902</v>
+        <v>336.4885879134903</v>
       </c>
       <c r="E74" s="2" t="n">
         <v>0</v>
@@ -4368,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>22.744141254236</v>
+        <v>22.7441412508397</v>
       </c>
       <c r="I74" s="2" t="n">
         <v>13.55322218679654</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-6.784374089768653</v>
+        <v>-6.784374089665615</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>326.3259631154089</v>
+        <v>326.3259631154091</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>339</v>
@@ -4421,7 +4421,7 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>46.76206032428988</v>
+        <v>46.76206034004523</v>
       </c>
       <c r="I75" s="2" t="n">
         <v>14.10348838068576</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.614453599047204</v>
+        <v>0.6144535978107966</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>325.2851315812709</v>
+        <v>325.285131581271</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>31.7</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>47.16631368017756</v>
+        <v>47.16631363884852</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>10.73152052963081</v>
+        <v>10.7315205630236</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.4294577746412609</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.110567617736008</v>
+        <v>0.1105676178493454</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>44.44805461974764</v>
+        <v>44.4480544827124</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>31.21094893079531</v>
+        <v>31.2109489699174</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.3512186134349756</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.0379538064814788</v>
+        <v>0.0379538065742046</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,7 +4580,7 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>52.45162463666723</v>
+        <v>52.45162467694738</v>
       </c>
       <c r="I78" s="2" t="n">
         <v>14.55947655572952</v>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>50.57773566148779</v>
+        <v>50.57773563833131</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>7.257360383668404</v>
+        <v>7.257360392659241</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.6661512903597218</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.2075581291819326</v>
+        <v>0.2075581292643527</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>314.6822596324323</v>
+        <v>314.6822596324353</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>41.4</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>48.26589306490867</v>
+        <v>48.2658929841552</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.76683271620594</v>
+        <v>14.76683294990132</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.5766456645155267</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.1445446853842949</v>
+        <v>0.1445446856109555</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>49.22567739110686</v>
+        <v>49.22567757025753</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>20.526862358174</v>
+        <v>20.52686237863223</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.3713511181953478</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.08386726228336119</v>
+        <v>-0.08386726242759809</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>305.2992925314886</v>
+        <v>305.2992925314885</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>308</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>34.6551055957385</v>
+        <v>34.65510571984376</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>18.94289073758593</v>
+        <v>18.94289079410513</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.553879515322136</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.5548210589467941</v>
+        <v>-0.5548210590498721</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>43.07493393738001</v>
+        <v>43.0749340747703</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>22.20946148401374</v>
+        <v>22.20946149350726</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.5523699655991354</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>1.379913999118092</v>
+        <v>1.379913999221106</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>296.3890237427447</v>
+        <v>296.3890237427446</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>105.5</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>40.230250677799</v>
+        <v>40.23025053587533</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>30.56240190731183</v>
+        <v>30.56240196367884</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.3751726085507562</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.3019429064427252</v>
+        <v>0.301942906957878</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>43.15925123171807</v>
+        <v>43.15925120605355</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>22.49913982661285</v>
+        <v>22.4991398346705</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.9073192493865792</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>-0.0190330549748827</v>
+        <v>-0.0190330549542787</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -5007,7 +5007,7 @@
         <v>44.18807598875662</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>19.26412130227236</v>
+        <v>19.26412148203671</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.3541290154393221</v>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>285.3140611042817</v>
+        <v>285.3140611042815</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>497.5</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>35.77600727306255</v>
+        <v>35.77600730245919</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>19.36962392160269</v>
+        <v>19.36962393794899</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>1.299959963630846</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-3.009661927923279</v>
+        <v>-3.00966192864442</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.97292386915528</v>
+        <v>50.9729238509125</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>10.47522095962943</v>
+        <v>10.47522098451468</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.3404588542382195</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0530873819297436</v>
+        <v>0.0530873820739832</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5149,7 +5149,7 @@
         <v/>
       </c>
       <c r="D89" s="2" t="n">
-        <v>276.0272996182998</v>
+        <v>276.0272996182997</v>
       </c>
       <c r="E89" s="2" t="n">
         <v>52.2</v>
@@ -5166,7 +5166,7 @@
         <v>42.33340835768306</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>17.4593494405147</v>
+        <v>17.45934951510271</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.7892652920150328</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.080329916715</v>
+        <v>0.0803299167974246</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>34.45714689812839</v>
+        <v>34.45714701820974</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>25.79794638101352</v>
+        <v>25.79794650492025</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.114153935332259</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.1714303616007788</v>
+        <v>0.1714303616832024</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>271.6555538138811</v>
+        <v>271.6555538138812</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>544</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>42.86408147948162</v>
+        <v>42.86408153282374</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>19.14862916092046</v>
+        <v>19.1486292474251</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.2470674217949016</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-5.415859469599446</v>
+        <v>-5.415859472072087</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5308,7 +5308,7 @@
         <v/>
       </c>
       <c r="D92" s="2" t="n">
-        <v>270.5999798672033</v>
+        <v>270.5999798672032</v>
       </c>
       <c r="E92" s="2" t="n">
         <v>41.5</v>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>44.96463798742708</v>
+        <v>44.96463802953522</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>9.98480364937123</v>
+        <v>9.984803650289273</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.6339514851264199</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.0047222831767486</v>
+        <v>-0.0047222832179571</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>269.865032112222</v>
+        <v>269.8650321122238</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>31.3</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>53.05423401603606</v>
+        <v>53.05423411080766</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>13.66877378453562</v>
+        <v>13.66877385190435</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.9055235590934892</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.1171173646097306</v>
+        <v>0.1171173646818504</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>268.0281521949976</v>
+        <v>268.0281521949975</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>74</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>41.07839210247571</v>
+        <v>41.07839183532043</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>12.15370789091294</v>
+        <v>12.15370813823671</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.4736994699117967</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.0388264424854908</v>
+        <v>-0.0388264420733741</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>262.6207978429107</v>
+        <v>262.6207978429106</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>49.9</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>53.63598499903493</v>
+        <v>53.63598500570047</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>15.14886839493266</v>
+        <v>15.14886841168128</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.4046483994907485</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.42518194949988</v>
+        <v>0.4251819494380582</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>34.01757260059605</v>
+        <v>34.01757269714639</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>24.62446444756339</v>
+        <v>24.62446447111283</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.9452214486096776</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.5309518754120593</v>
+        <v>-0.5309518755356953</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>49.63415193374427</v>
+        <v>49.63415214643608</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>11.9631397783371</v>
+        <v>11.96313978250093</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.6413841958486479</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>1.231988687229399</v>
+        <v>1.231988686508194</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>253.1369387098765</v>
+        <v>253.1369387098768</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>127</v>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>50.1166516167295</v>
+        <v>50.11665163793928</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.22637093858975</v>
+        <v>19.22637082989426</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.2399527825461679</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>1.842823825691052</v>
+        <v>1.842823824763795</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>45.3278077827737</v>
+        <v>45.32780774924314</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>14.65112930704046</v>
+        <v>14.65112930809184</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.7447265059150433</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.0546517431019008</v>
+        <v>0.0546517432358346</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>51.87822312094049</v>
+        <v>51.87822316426746</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>12.54117167720771</v>
+        <v>12.54117168971925</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.4192368538558683</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.2453664315215517</v>
+        <v>0.2453664314803415</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>237.9365651786588</v>
+        <v>237.9365651786589</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>22.85</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>46.59610595219369</v>
+        <v>46.5961060312595</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>16.02657628197688</v>
+        <v>16.02657632655314</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.2660974403330715</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.0069184787249843</v>
+        <v>0.006918478683775</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>36.21181957119524</v>
+        <v>36.21181943543718</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>25.88483923653997</v>
+        <v>25.8848394309502</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>0.2871225570612074</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.2950506653978304</v>
+        <v>-0.2950506651093518</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>221.3037912671374</v>
+        <v>221.3037912671372</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>0</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>27.48900268164485</v>
+        <v>27.48900268753954</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>16.63191174043483</v>
+        <v>16.63191183750586</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-1.617384178180838</v>
+        <v>-1.617384178139626</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>51.00187790599437</v>
+        <v>51.00187790428424</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>9.582401092731963</v>
+        <v>9.582401048164582</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.5925048141016146</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>0.2686487729916374</v>
+        <v>0.2686487730019397</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>219.7508490207583</v>
+        <v>219.7508490207584</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>31</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>40.42759491338485</v>
+        <v>40.42759522567731</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>16.12340705508657</v>
+        <v>16.12340717189815</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.9712822687170788</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.0664060498333652</v>
+        <v>-0.06640604988487921</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>40.64570616192421</v>
+        <v>40.64570655143384</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.72310009198448</v>
+        <v>16.72310016194607</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.3842965200795153</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0563361937268678</v>
+        <v>0.0563361940359659</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,7 +6117,7 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>42.39926394223667</v>
+        <v>42.39926394793338</v>
       </c>
       <c r="I107" s="2" t="n">
         <v>17.88937333038178</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.042079592512491</v>
+        <v>0.042079592498069</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>41.18486409559488</v>
+        <v>41.18486397076366</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>25.17777558034955</v>
+        <v>25.17777581015171</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.1560370124023627</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.2439083003529663</v>
+        <v>0.2439083008681148</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>210.5071497297923</v>
+        <v>210.5071497297922</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>68.7</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>52.50052029878268</v>
+        <v>52.50052028722487</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>7.284511590446956</v>
+        <v>7.284511759853149</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.7663444135434601</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>3.511323959237629</v>
+        <v>3.511323960267912</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>49.8496279324039</v>
+        <v>49.84962794849375</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>14.96897815367396</v>
+        <v>14.96897802550654</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.340937166016628</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.1332983695917149</v>
+        <v>0.1332983693856485</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>42.96360605585787</v>
+        <v>42.96360611680451</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>13.65012182903726</v>
+        <v>13.65012188801317</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.3492694072126049</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-3.072055940667806</v>
+        <v>-3.072055937577112</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.64299573042736</v>
+        <v>44.6429955097758</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>11.33901573914276</v>
+        <v>11.33901589869094</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.171532096810977</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1894128229206506</v>
+        <v>-0.1894128214576416</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>51.35035179271367</v>
+        <v>51.35035177071</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>15.03185936351223</v>
+        <v>15.03185935933276</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.4292346496648372</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.5900059867765262</v>
+        <v>0.590005986673495</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6474,7 +6474,7 @@
         <v/>
       </c>
       <c r="D114" s="2" t="n">
-        <v>201.4612923828052</v>
+        <v>201.4612923828062</v>
       </c>
       <c r="E114" s="2" t="n">
         <v>32.45</v>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>45.09518514390973</v>
+        <v>45.09518525138712</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>19.47250754246654</v>
+        <v>19.47250757803604</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.3841622350083522</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0332903888749848</v>
+        <v>0.0332903888543798</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>201.3622389803221</v>
+        <v>201.3622389803224</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>58.8</v>
@@ -6541,7 +6541,7 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>41.57073606203335</v>
+        <v>41.5707361993773</v>
       </c>
       <c r="I115" s="2" t="n">
         <v>15.21822528847986</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1784904209350925</v>
+        <v>-0.1784904211411517</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.76733160827698</v>
+        <v>39.76733161682601</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>14.19198676057521</v>
+        <v>14.19198682046007</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.6646540163261692</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-103.6076043019293</v>
+        <v>-103.6076043101722</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>44.64011737792781</v>
+        <v>44.64011769358486</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>17.95638213676783</v>
+        <v>17.95638218800901</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.4594244036317838</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.07015206314359521</v>
+        <v>0.0701520634526772</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>163.1362691119624</v>
+        <v>163.1362691119623</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>214</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>40.6331860265698</v>
+        <v>40.6331859742882</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>23.83361604241929</v>
+        <v>23.83361609181967</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.4603245019449106</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>1.755236778664827</v>
+        <v>1.755236778767847</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,7 +6753,7 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>40.19107123827547</v>
+        <v>40.19107130303673</v>
       </c>
       <c r="I119" s="2" t="n">
         <v>18.90451298494492</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-1.140880203825823</v>
+        <v>-1.140880203928835</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6809,7 +6809,7 @@
         <v>40.67576528381733</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>10.32187127600676</v>
+        <v>10.32187124278139</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.4807071250994642</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>35.93313347893019</v>
+        <v>35.93313370998274</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>14.42531063165845</v>
+        <v>14.42531088453532</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.5912643743928939</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.032944566926695</v>
+        <v>-0.0329445668122498</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>39.42566515940095</v>
+        <v>39.42566513308714</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>16.00938919368577</v>
+        <v>16.00938919368576</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.7665949264223837</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0026604641920382</v>
+        <v>-0.0026604641302202</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>36.12839456097191</v>
+        <v>36.12839490395181</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>18.83398914984016</v>
+        <v>18.83398912186306</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.5171171932398859</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.2774329459747289</v>
+        <v>-0.2774329463868292</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>52.40256147282226</v>
+        <v>52.40256113611493</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>6.589316137819963</v>
+        <v>6.589316137835839</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.1717163096355722</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.6680866409190112</v>
+        <v>0.6680866409396138</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>45.49448725944038</v>
+        <v>45.49448746739471</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>14.33591618701237</v>
+        <v>14.33591616651753</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.3107575909571903</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.9009519552157856</v>
+        <v>0.9009519548036886</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>124.0154397632359</v>
+        <v>124.0154397632358</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>57.6</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>27.29818954425885</v>
+        <v>27.29818946411157</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>18.97000896903415</v>
+        <v>18.97000897750958</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>1.056226180281053</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.2484329955927415</v>
+        <v>-0.2484329955515352</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>45.04276452708238</v>
+        <v>45.04276454418875</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>12.73002416304794</v>
+        <v>12.73002418027572</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.3409157264369457</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>0.1591318837820872</v>
+        <v>0.1591318839263277</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
scan: seg6 2026-09-29 00:37 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq7_2026-09-24.xlsx
+++ b/output/full_scan/batch_seq7_2026-09-24.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>68.66754019650855</v>
+        <v>68.66754018931618</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>26.83106218996431</v>
+        <v>26.83106213948439</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>2.685524105208017</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.957899931099302</v>
+        <v>1.957899930988008</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>71.16375683481112</v>
+        <v>71.1637567869612</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>21.7431787825884</v>
+        <v>21.743178741203</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.661943371713502</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.1545851918439826</v>
+        <v>0.1545851918662406</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>58.27249355224106</v>
+        <v>58.27249349729385</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>7.932196171050655</v>
+        <v>7.932196184984674</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>8.584258392238151</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.2035670185769997</v>
+        <v>0.2035670189664433</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>65.27530100318893</v>
+        <v>65.27530100488829</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>17.43169736750527</v>
+        <v>17.43169730553124</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>4.346659824971685</v>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>61.79438103867085</v>
+        <v>61.79438092567332</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>22.3094471552436</v>
+        <v>22.30944712063054</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>3.17558471647802</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>1.427628112087846</v>
+        <v>1.427628112755487</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>64.70178542397032</v>
+        <v>64.7017854170779</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>30.19848254674888</v>
+        <v>30.19848247750832</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>0.97728597061346</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>1.838392146546833</v>
+        <v>1.838392146624721</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>82.4614763644873</v>
+        <v>82.4614763354798</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>26.41998847705492</v>
+        <v>26.41998855725634</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>3.207844850229248</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>22.12763056310636</v>
+        <v>22.12763056444162</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>68.75851760375002</v>
+        <v>68.75851750334304</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>23.01777665367185</v>
+        <v>23.01777675408971</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>4.296995099878581</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>10.01171512533824</v>
+        <v>10.01171512667349</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>56.24096104817474</v>
+        <v>56.2409610490765</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>10.98468357032213</v>
+        <v>10.98468368483788</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>0.8603444852936751</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>0.2404680369317802</v>
+        <v>0.240468034038745</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>60.50713018306762</v>
+        <v>60.5071302006708</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>37.95936948238987</v>
+        <v>37.95936953241894</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>0.650772025543959</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>-0.257228923350441</v>
+        <v>-0.2572289233949609</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>63.31977517961854</v>
+        <v>63.31977520631171</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>45.20069381244598</v>
+        <v>45.20069383039493</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.4302284329160745</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>0.2442435272146399</v>
+        <v>0.2442435271256213</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v/>
       </c>
       <c r="D13" s="2" t="n">
-        <v>848.6490266520972</v>
+        <v>848.6490266520968</v>
       </c>
       <c r="E13" s="2" t="n">
         <v>667</v>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>58.35151317067923</v>
+        <v>58.35151314743455</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>16.3956978809125</v>
+        <v>16.39569785870655</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.365708007827902</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>7.9234483538298</v>
+        <v>7.923448355498925</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>60.54223831820774</v>
+        <v>60.54223819673126</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>28.12260914673256</v>
+        <v>28.1226091689872</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>0.4464859771818252</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>1.571134811813875</v>
+        <v>1.571134813260405</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>65.61060064388079</v>
+        <v>65.61060065429317</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>32.15373259400138</v>
+        <v>32.15373255862614</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>0.6827230607894571</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>26.13903972292927</v>
+        <v>26.13903972604473</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>59.67954326340881</v>
+        <v>59.67954323679551</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>31.81749372378981</v>
+        <v>31.81749372030224</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>0.6040651995779337</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.0411138574531673</v>
+        <v>0.0411138575644391</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1347,10 +1347,10 @@
         <v>0</v>
       </c>
       <c r="H17" s="2" t="n">
-        <v>62.55096454979986</v>
+        <v>62.55096456957175</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>44.75207661328924</v>
+        <v>44.752076615066</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.4966982704420574</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>0.4467829364482902</v>
+        <v>0.4467829364705387</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>67.16033985970495</v>
+        <v>67.16033985120029</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>62.49451583781153</v>
+        <v>62.49451593010431</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.149941419890234</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2.941039513748819</v>
+        <v>2.941039514260673</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>741.7553124543483</v>
+        <v>741.7553124543472</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>261.5</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>65.14607035151424</v>
+        <v>65.14607021839537</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>37.45305625220068</v>
+        <v>37.45305624422762</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>0.5241372274217474</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>2.498773222618782</v>
+        <v>2.498773224399156</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>56.57339564812207</v>
+        <v>56.57339565370091</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>21.00564400756689</v>
+        <v>21.00564420152987</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>0.5684408896010303</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>14.32666916301569</v>
+        <v>14.32666916223681</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>54.79130147505931</v>
+        <v>54.79130140925704</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>30.71886418578853</v>
+        <v>30.71886426459456</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>0.7554779489056903</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>1.482179918975275</v>
+        <v>1.482179920088005</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>72.06436274263918</v>
+        <v>72.06436270604425</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>30.08730806053153</v>
+        <v>30.08730806678129</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>0.8183871815292657</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.2901901869433685</v>
+        <v>0.2901901869211133</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>52.31573324599304</v>
+        <v>52.31573294263024</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>7.777975798880761</v>
+        <v>7.777975326956708</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.521466971058252</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>0.07855370498717219</v>
+        <v>0.0785537203648676</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>679.5983977201183</v>
+        <v>679.5983977201184</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>143</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>55.35700630691913</v>
+        <v>55.35700617513169</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>43.08147161332783</v>
+        <v>43.08147165483943</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.3510109837704807</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>0.8499582277029791</v>
+        <v>0.8499582291717562</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1771,10 +1771,10 @@
         <v>0</v>
       </c>
       <c r="H25" s="2" t="n">
-        <v>25.59756300519639</v>
+        <v>25.59756296785276</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>45.21174388568553</v>
+        <v>45.21174385601048</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.8078270744650331</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>17.01331214545746</v>
+        <v>17.01331216993674</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,7 +1824,7 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>62.55632771123713</v>
+        <v>62.55632768482751</v>
       </c>
       <c r="I26" s="2" t="n">
         <v>23.88546752293477</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>1.329744655861554</v>
+        <v>1.329744655906063</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>67.57478715438286</v>
+        <v>67.57478714892892</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>40.2453613602517</v>
+        <v>40.24536136025171</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>1.972543201921374</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>1.135904391213288</v>
+        <v>1.135904391013</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>51.16607896205471</v>
+        <v>51.16607900554012</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>23.07965741739384</v>
+        <v>23.07965742592058</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.6587897239350179</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>-0.6874192281964873</v>
+        <v>-0.6874192287528496</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1969,7 +1969,7 @@
         <v/>
       </c>
       <c r="D29" s="2" t="n">
-        <v>604.2253956784633</v>
+        <v>604.2253956784632</v>
       </c>
       <c r="E29" s="2" t="n">
         <v>358.5</v>
@@ -1983,10 +1983,10 @@
         <v>0</v>
       </c>
       <c r="H29" s="2" t="n">
-        <v>56.5849993229416</v>
+        <v>56.58499930785391</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>10.2918834106784</v>
+        <v>10.29188342109712</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>0.8317529702446623</v>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>52.09765784986006</v>
+        <v>52.09765771682353</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>23.18118076870248</v>
+        <v>23.18118077294859</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>0.3336766004557814</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>-0.9119035856693758</v>
+        <v>-0.9119035818861896</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2089,10 +2089,10 @@
         <v>0</v>
       </c>
       <c r="H31" s="2" t="n">
-        <v>47.39828998574609</v>
+        <v>47.39828995142768</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>27.40172094996863</v>
+        <v>27.40172090657838</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.392094524945494</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>-1.27349919113004</v>
+        <v>-1.273499190651565</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>51.68650901865525</v>
+        <v>51.68650903663533</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>33.13407067885349</v>
+        <v>33.13407067200448</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.9088189620361444</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-14.34582857827348</v>
+        <v>-14.34582856825892</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2198,7 +2198,7 @@
         <v>55.88810671340467</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>21.93956159338195</v>
+        <v>21.93956157852659</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>1.663121215559225</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>0.3309913466457752</v>
+        <v>0.3309913468015817</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2234,7 +2234,7 @@
         <v/>
       </c>
       <c r="D34" s="2" t="n">
-        <v>567.567825044792</v>
+        <v>567.5678250447919</v>
       </c>
       <c r="E34" s="2" t="n">
         <v>179</v>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>57.78139645137507</v>
+        <v>57.78139637244322</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>16.6423997007581</v>
+        <v>16.64239973701356</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>1.409581288192835</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>0.577174022834082</v>
+        <v>0.5771740230343827</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>58.52992308126178</v>
+        <v>58.52992305910213</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>31.80823287534841</v>
+        <v>31.8082328651986</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>0.3625300479778954</v>
@@ -2340,7 +2340,7 @@
         <v/>
       </c>
       <c r="D36" s="2" t="n">
-        <v>532.8771635878538</v>
+        <v>532.8771635878549</v>
       </c>
       <c r="E36" s="2" t="n">
         <v>42</v>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>55.36330474930742</v>
+        <v>55.3633049456635</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>21.72365924050072</v>
+        <v>21.72365942023316</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.304760356772791</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.0603378433968663</v>
+        <v>-0.060337843530395</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>31.69503153248954</v>
+        <v>31.69502468910697</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>32.59321928795873</v>
+        <v>32.59322336563498</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>2.013053626871306</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>0.4112821095165779</v>
+        <v>0.4112821326881848</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>55.785844708163</v>
+        <v>55.78584468641977</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>9.630348031654968</v>
+        <v>9.630348084029132</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.4155415414568079</v>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>52.60058351316243</v>
+        <v>52.60058349494181</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>8.975604874723546</v>
+        <v>8.975604810447029</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.7337314238331761</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.0452549454591612</v>
+        <v>0.0452549455370523</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2622,7 +2622,7 @@
         <v>54.03842997062653</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>25.32562451096538</v>
+        <v>25.32562446195569</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.2435764880321545</v>
@@ -2637,7 +2637,7 @@
         <v>-1</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>-0.5147660984946953</v>
+        <v>-0.5147660983166582</v>
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
@@ -2658,7 +2658,7 @@
         <v/>
       </c>
       <c r="D42" s="2" t="n">
-        <v>503.5177132338882</v>
+        <v>503.5177132338883</v>
       </c>
       <c r="E42" s="2" t="n">
         <v>540</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>52.96310899466217</v>
+        <v>52.96310896706731</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>27.72772531839418</v>
+        <v>27.72772514293023</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.4416483554075971</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-7.160934445296718</v>
+        <v>-7.160934443961388</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>48.37480316821787</v>
+        <v>48.3748031560292</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>13.99015890846122</v>
+        <v>13.99015891206445</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>0.4652378730945042</v>
@@ -2743,7 +2743,7 @@
         <v>-1</v>
       </c>
       <c r="N43" s="2" t="n">
-        <v>0.8010099711968843</v>
+        <v>0.801009971330422</v>
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="D44" s="2" t="n">
-        <v>485.4243133896993</v>
+        <v>485.4243133896994</v>
       </c>
       <c r="E44" s="2" t="n">
         <v>86.59999999999999</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>61.13659915155117</v>
+        <v>61.13659909668336</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>19.10493708206357</v>
+        <v>19.10493711985196</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>1.136273133488234</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>1.105702871333707</v>
+        <v>1.105702871467231</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>47.36817246581801</v>
+        <v>47.36817253927163</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>25.33728966958646</v>
+        <v>25.33728967738845</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.4657350026052051</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>-0.0040183611321781</v>
+        <v>-0.0040183611099199</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2870,7 +2870,7 @@
         <v/>
       </c>
       <c r="D46" s="2" t="n">
-        <v>455.8431542223494</v>
+        <v>455.8431542223491</v>
       </c>
       <c r="E46" s="2" t="n">
         <v>51.4</v>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>55.49458303328909</v>
+        <v>55.49458289336413</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>18.3449867841258</v>
+        <v>18.34498682984626</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>1.207504683192515</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>0.4618526015663274</v>
+        <v>0.4618526018111248</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>42.24014344628299</v>
+        <v>42.24014342946501</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>21.67275727779379</v>
+        <v>21.67275724973222</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>0.5335609419929919</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>-23.92442063197018</v>
+        <v>-23.92442063219265</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>54.8224720189723</v>
+        <v>54.82247201029238</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>46.55901904509773</v>
+        <v>46.5590190241526</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>0.1434060592326219</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>-0.1279232031604884</v>
+        <v>-0.1279232031827342</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>52.12765402325228</v>
+        <v>52.12765400882616</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>8.456619753008512</v>
+        <v>8.456619681989764</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>1.324830518212111</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>0.0971265220804132</v>
+        <v>0.09712652223619329</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>50.43995570404039</v>
+        <v>50.43995561232988</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>22.54481023784425</v>
+        <v>22.5448102834015</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.531165319874093</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.0915255370728533</v>
+        <v>-0.09152553687256711</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3135,7 +3135,7 @@
         <v/>
       </c>
       <c r="D51" s="2" t="n">
-        <v>423.3575384551401</v>
+        <v>423.3575384551402</v>
       </c>
       <c r="E51" s="2" t="n">
         <v>51.3</v>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>45.13497129517609</v>
+        <v>45.13497128111819</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>13.50937649122115</v>
+        <v>13.50937651785586</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.647273987081031</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>0.0385486183857277</v>
+        <v>0.0385486183968639</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3188,7 +3188,7 @@
         <v/>
       </c>
       <c r="D52" s="2" t="n">
-        <v>418.6943569607691</v>
+        <v>418.6943569607688</v>
       </c>
       <c r="E52" s="2" t="n">
         <v>948</v>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>49.47095741242141</v>
+        <v>49.47095737078124</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>8.444011691681018</v>
+        <v>8.444011644302291</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.93264437588126</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>4.940413010902663</v>
+        <v>4.94041301312808</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3241,7 +3241,7 @@
         <v/>
       </c>
       <c r="D53" s="2" t="n">
-        <v>418.2524790326087</v>
+        <v>418.2524790326088</v>
       </c>
       <c r="E53" s="2" t="n">
         <v>465.5</v>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>53.86008532407225</v>
+        <v>53.86008528287902</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>12.19947711498095</v>
+        <v>12.19947709535342</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.5959109105149348</v>
@@ -3308,10 +3308,10 @@
         <v>0</v>
       </c>
       <c r="H54" s="2" t="n">
-        <v>53.40412464597301</v>
+        <v>53.40412457652513</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>19.310935800471</v>
+        <v>19.3109358485961</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.6476801554183461</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.9186962190156338</v>
+        <v>0.9186962195719944</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3347,7 +3347,7 @@
         <v/>
       </c>
       <c r="D55" s="2" t="n">
-        <v>409.3218640015364</v>
+        <v>409.3218640015365</v>
       </c>
       <c r="E55" s="2" t="n">
         <v>90.5</v>
@@ -3364,7 +3364,7 @@
         <v>44.72886892065956</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>10.1847946646186</v>
+        <v>10.18479466966998</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>1.505333590988018</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>0.0176562705992771</v>
+        <v>0.0176562704434968</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3400,7 +3400,7 @@
         <v/>
       </c>
       <c r="D56" s="2" t="n">
-        <v>404.8845594177957</v>
+        <v>404.884559417796</v>
       </c>
       <c r="E56" s="2" t="n">
         <v>24.5</v>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>49.60827128143913</v>
+        <v>49.60827159887207</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>26.15023116888705</v>
+        <v>26.15023116772975</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.8650145154211294</v>
@@ -3432,7 +3432,7 @@
         <v>-1</v>
       </c>
       <c r="N56" s="2" t="n">
-        <v>0.1837762696252162</v>
+        <v>0.1837762696363426</v>
       </c>
       <c r="O56" s="2" t="inlineStr">
         <is>
@@ -3453,7 +3453,7 @@
         <v/>
       </c>
       <c r="D57" s="2" t="n">
-        <v>402.7111623172892</v>
+        <v>402.7111623172921</v>
       </c>
       <c r="E57" s="2" t="n">
         <v>44.2</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>55.11978952310063</v>
+        <v>55.11978934212041</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>29.06923083260857</v>
+        <v>29.06923140667173</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.40320428304767</v>
@@ -3485,7 +3485,7 @@
         <v>-1</v>
       </c>
       <c r="N57" s="2" t="n">
-        <v>0.4088516819230153</v>
+        <v>0.4088516827241663</v>
       </c>
       <c r="O57" s="2" t="inlineStr">
         <is>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>402.3567160515287</v>
+        <v>402.3567160515306</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>1110</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>50.70385319998633</v>
+        <v>50.70385322102788</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>11.18590270123124</v>
+        <v>11.18590273826572</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>0.4290261573668845</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>-10.5229922432542</v>
+        <v>-10.52299223924853</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3559,7 +3559,7 @@
         <v/>
       </c>
       <c r="D59" s="2" t="n">
-        <v>397.5606799965664</v>
+        <v>397.5606799965663</v>
       </c>
       <c r="E59" s="2" t="n">
         <v>22.65</v>
@@ -3573,7 +3573,7 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>50.32722816895669</v>
+        <v>50.32722815754747</v>
       </c>
       <c r="I59" s="2" t="n">
         <v>8.989604692640697</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.2458652135816548</v>
+        <v>0.2458652136372933</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>54.97217806375415</v>
+        <v>54.972178066211</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>17.02854771431543</v>
+        <v>17.02854770067713</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.03301322482184</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-6.705685453196642</v>
+        <v>-6.705685451394034</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>382.4710173027301</v>
+        <v>382.4710173027298</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>32.8</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>50.1742358134637</v>
+        <v>50.17423562083926</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>23.30150391297365</v>
+        <v>23.30150403241839</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>0.323416615282644</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>-0.0883854448550398</v>
+        <v>-0.0883854444767171</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3718,7 +3718,7 @@
         <v/>
       </c>
       <c r="D62" s="2" t="n">
-        <v>378.2401478543658</v>
+        <v>378.2401478543657</v>
       </c>
       <c r="E62" s="2" t="n">
         <v>46.65</v>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>34.96315223405169</v>
+        <v>34.96315224549721</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>31.58515635258613</v>
+        <v>31.58515631791143</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.3319491119899236</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-0.0625534501077995</v>
+        <v>-0.06255345013005879</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>48.15406298716601</v>
+        <v>48.15406299112529</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>23.04032668827005</v>
+        <v>23.04032661603983</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.2955256328703418</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>-2.332987316002886</v>
+        <v>-2.332987316025161</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>45.9269171851949</v>
+        <v>45.92691716778028</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>16.52135472293203</v>
+        <v>16.52135467846428</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>0.5972748766961367</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.0746118402771541</v>
+        <v>-0.07461184022151759</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="D65" s="2" t="n">
-        <v>369.5997760213101</v>
+        <v>369.59977602131</v>
       </c>
       <c r="E65" s="2" t="n">
         <v>97.5</v>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>49.0284220944752</v>
+        <v>49.02842190301805</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>9.539050306776504</v>
+        <v>9.539050302196358</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>0.6590440111141078</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>-0.0245580212044544</v>
+        <v>-0.0245580207816215</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>43.52159340238235</v>
+        <v>43.52159346753374</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>11.4136409625665</v>
+        <v>11.41364097543487</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>0.3222677259872201</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>-0.1885271147649017</v>
+        <v>-0.1885271140972693</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,7 +3997,7 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>40.46448163914612</v>
+        <v>40.464481343229</v>
       </c>
       <c r="I67" s="2" t="n">
         <v>12.83135036525853</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-0.2613456663638074</v>
+        <v>-0.2613456655403907</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>57.2558986250877</v>
+        <v>57.25589854083006</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>19.98805306399838</v>
+        <v>19.98805305109872</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.9463948142694908</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>1.217486811777785</v>
+        <v>1.217486812334147</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4089,7 +4089,7 @@
         <v/>
       </c>
       <c r="D69" s="2" t="n">
-        <v>348.3542541384186</v>
+        <v>348.3542541384185</v>
       </c>
       <c r="E69" s="2" t="n">
         <v>71.3</v>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>46.92396406438479</v>
+        <v>46.92396402893549</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>13.88576413953373</v>
+        <v>13.88576406430952</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.5174383721506689</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>0.044486684353754</v>
+        <v>0.0444866845095468</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4142,7 +4142,7 @@
         <v/>
       </c>
       <c r="D70" s="2" t="n">
-        <v>346.2635521145977</v>
+        <v>346.263552114599</v>
       </c>
       <c r="E70" s="2" t="n">
         <v>60.1</v>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>46.2396751519973</v>
+        <v>46.23967502169271</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>25.60654187287011</v>
+        <v>25.60654196184609</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.5507151254854856</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>0.2183728885774385</v>
+        <v>0.2183728890225302</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>57.41756283461797</v>
+        <v>57.41756270518815</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>19.91919289890828</v>
+        <v>19.9191929687957</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.6419259175666775</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.5351916854884915</v>
+        <v>0.5351916856887857</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>44.69811224540418</v>
+        <v>44.69811224174484</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>13.70076773373744</v>
+        <v>13.70076771563081</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>0.366188600864838</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>-3.595449208921471</v>
+        <v>-3.595449208587653</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>53.39391177200346</v>
+        <v>53.3939122155664</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>15.04376320296989</v>
+        <v>15.04376316973749</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.7440767050085816</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.186589495420639</v>
+        <v>0.1865894954540216</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>22.7441412508397</v>
+        <v>22.74414125167158</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>13.55322218679654</v>
+        <v>13.55322226404363</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>7.223502387367539e-05</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>-6.784374089665615</v>
+        <v>-6.7843740897769</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4407,7 +4407,7 @@
         <v/>
       </c>
       <c r="D75" s="2" t="n">
-        <v>326.3259631154091</v>
+        <v>326.3259631154089</v>
       </c>
       <c r="E75" s="2" t="n">
         <v>339</v>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>46.76206034004523</v>
+        <v>46.76206048022344</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>14.10348838068576</v>
+        <v>14.10348840664546</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.2578538644573807</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>0.6144535978107966</v>
+        <v>0.6144535969206393</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>325.285131581271</v>
+        <v>325.2851315812711</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>31.7</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>47.16631363884852</v>
+        <v>47.1663135680051</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>10.7315205630236</v>
+        <v>10.73152062215036</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.4294577746412609</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>0.1105676178493454</v>
+        <v>0.1105676178938529</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>44.4480544827124</v>
+        <v>44.44805456704177</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>31.2109489699174</v>
+        <v>31.2109490778978</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>0.3512186134349756</v>
@@ -4545,7 +4545,7 @@
         <v>-1</v>
       </c>
       <c r="N77" s="2" t="n">
-        <v>0.0379538065742046</v>
+        <v>0.0379538065964585</v>
       </c>
       <c r="O77" s="2" t="inlineStr">
         <is>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>52.45162467694738</v>
+        <v>52.45162408327221</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>14.55947655572952</v>
+        <v>14.55947660341976</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.4059001519848108</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>0.1592680305791799</v>
+        <v>0.1592680308017234</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>50.57773563833131</v>
+        <v>50.57773648621435</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>7.257360392659241</v>
+        <v>7.257360402165956</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.6661512903597218</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>0.2075581292643527</v>
+        <v>0.2075581293088619</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4672,7 +4672,7 @@
         <v/>
       </c>
       <c r="D80" s="2" t="n">
-        <v>314.6822596324353</v>
+        <v>314.6822596324315</v>
       </c>
       <c r="E80" s="2" t="n">
         <v>41.4</v>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>48.2658929841552</v>
+        <v>48.26589262912802</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>14.76683294990132</v>
+        <v>14.76683310251186</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.5766456645155267</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.1445446856109555</v>
+        <v>0.1445446857667398</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>49.22567757025753</v>
+        <v>49.2256773413321</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>20.52686237863223</v>
+        <v>20.52686234643453</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>0.3713511181953478</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>-0.08386726242759809</v>
+        <v>-0.08386726211604199</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4778,7 +4778,7 @@
         <v/>
       </c>
       <c r="D82" s="2" t="n">
-        <v>305.2992925314885</v>
+        <v>305.2992925314887</v>
       </c>
       <c r="E82" s="2" t="n">
         <v>308</v>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>34.65510571984376</v>
+        <v>34.65510543662472</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>18.94289079410513</v>
+        <v>18.94289082656574</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.553879515322136</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.5548210590498721</v>
+        <v>-0.5548210581596313</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>43.0749340747703</v>
+        <v>43.07493379005993</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>22.20946149350726</v>
+        <v>22.20946166730726</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.5523699655991354</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>1.379913999221106</v>
+        <v>1.379914001001452</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4884,7 +4884,7 @@
         <v/>
       </c>
       <c r="D84" s="2" t="n">
-        <v>296.3890237427446</v>
+        <v>296.3890237427447</v>
       </c>
       <c r="E84" s="2" t="n">
         <v>105.5</v>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>40.23025053587533</v>
+        <v>40.23025034134822</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>30.56240196367884</v>
+        <v>30.56240197970018</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.3751726085507562</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>0.301942906957878</v>
+        <v>0.3019429067353512</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>43.15925120605355</v>
+        <v>43.15925118506743</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>22.4991398346705</v>
+        <v>22.49913973025586</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>0.9073192493865792</v>
@@ -5004,7 +5004,7 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>44.18807598875662</v>
+        <v>44.18807605500734</v>
       </c>
       <c r="I86" s="2" t="n">
         <v>19.26412148203671</v>
@@ -5043,7 +5043,7 @@
         <v/>
       </c>
       <c r="D87" s="2" t="n">
-        <v>285.3140611042815</v>
+        <v>285.3140611042825</v>
       </c>
       <c r="E87" s="2" t="n">
         <v>497.5</v>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>35.77600730245919</v>
+        <v>35.77600726961765</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>19.36962393794899</v>
+        <v>19.3696239281069</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>1.299959963630846</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-3.00966192864442</v>
+        <v>-3.009661927420463</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>50.9729238509125</v>
+        <v>50.97292380179734</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>10.47522098451468</v>
+        <v>10.47522089788808</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.3404588542382195</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>0.0530873820739832</v>
+        <v>0.0530873821852623</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>42.33340835768306</v>
+        <v>42.33340841084989</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>17.45934951510271</v>
+        <v>17.45934965267273</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.7892652920150328</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.0803299167974246</v>
+        <v>0.0803299168864427</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>273.993084653335</v>
+        <v>273.9930846533349</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>30.3</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>34.45714701820974</v>
+        <v>34.45714690064757</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>25.79794650492025</v>
+        <v>25.79794667917637</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>1.114153935332259</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>0.1714303616832024</v>
+        <v>0.1714303620170194</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5255,7 +5255,7 @@
         <v/>
       </c>
       <c r="D91" s="2" t="n">
-        <v>271.6555538138812</v>
+        <v>271.6555538138811</v>
       </c>
       <c r="E91" s="2" t="n">
         <v>544</v>
@@ -5269,10 +5269,10 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>42.86408153282374</v>
+        <v>42.86408149766561</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>19.1486292474251</v>
+        <v>19.14862920301896</v>
       </c>
       <c r="J91" s="2" t="n">
         <v>0.2470674217949016</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-5.415859472072087</v>
+        <v>-5.415859470848043</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>44.96463802953522</v>
+        <v>44.96463795605668</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>9.984803650289273</v>
+        <v>9.984803677761256</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>0.6339514851264199</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-0.0047222832179571</v>
+        <v>-0.0047222831957071</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5361,7 +5361,7 @@
         <v/>
       </c>
       <c r="D93" s="2" t="n">
-        <v>269.8650321122238</v>
+        <v>269.8650321122221</v>
       </c>
       <c r="E93" s="2" t="n">
         <v>31.3</v>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>53.05423411080766</v>
+        <v>53.0542337873585</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>13.66877385190435</v>
+        <v>13.66877396654404</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.9055235590934892</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>0.1171173646818504</v>
+        <v>0.1171173648710093</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5414,7 +5414,7 @@
         <v/>
       </c>
       <c r="D94" s="2" t="n">
-        <v>268.0281521949975</v>
+        <v>268.0281521949976</v>
       </c>
       <c r="E94" s="2" t="n">
         <v>74</v>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>41.07839183532043</v>
+        <v>41.07839212302611</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>12.15370813823671</v>
+        <v>12.1537086040262</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.4736994699117967</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>-0.0388264420733741</v>
+        <v>-0.0388264421178838</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>53.63598500570047</v>
+        <v>53.6359849410961</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>15.14886841168128</v>
+        <v>15.14886843467086</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.4046483994907485</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>0.4251819494380582</v>
+        <v>0.4251819493935506</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>34.01757269714639</v>
+        <v>34.01757276575314</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>24.62446447111283</v>
+        <v>24.62446465744274</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.9452214486096776</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>-0.5309518755356953</v>
+        <v>-0.5309518754021758</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>49.63415214643608</v>
+        <v>49.63415204640566</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>11.96313978250093</v>
+        <v>11.9631399314347</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.6413841958486479</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>1.231988686508194</v>
+        <v>1.231988688288528</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>50.11665163793928</v>
+        <v>50.11665164299149</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>19.22637082989426</v>
+        <v>19.2263707562804</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>0.2399527825461679</v>
@@ -5693,10 +5693,10 @@
         <v>0</v>
       </c>
       <c r="H99" s="2" t="n">
-        <v>45.32780774924314</v>
+        <v>45.32780773242257</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>14.65112930809184</v>
+        <v>14.65112930452288</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.7447265059150433</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>0.0546517432358346</v>
+        <v>0.0546517432692177</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>51.87822316426746</v>
+        <v>51.87822312972204</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>12.54117168971925</v>
+        <v>12.54117166029528</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>0.4192368538558683</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.2453664314803415</v>
+        <v>0.2453664317028836</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v/>
       </c>
       <c r="D101" s="2" t="n">
-        <v>237.9365651786589</v>
+        <v>237.9365651786588</v>
       </c>
       <c r="E101" s="2" t="n">
         <v>22.85</v>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>46.5961060312595</v>
+        <v>46.59610596265779</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>16.02657632655314</v>
+        <v>16.02657633064856</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.2660974403330715</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>0.006918478683775</v>
+        <v>0.0069184786948979</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,7 +5852,7 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>36.21181943543718</v>
+        <v>36.21181947761693</v>
       </c>
       <c r="I102" s="2" t="n">
         <v>25.8848394309502</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.2950506651093518</v>
+        <v>-0.2950506653318996</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5891,7 +5891,7 @@
         <v/>
       </c>
       <c r="D103" s="2" t="n">
-        <v>221.3037912671372</v>
+        <v>221.3037912671373</v>
       </c>
       <c r="E103" s="2" t="n">
         <v>0</v>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>27.48900268753954</v>
+        <v>27.48900267960437</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>16.63191183750586</v>
+        <v>16.63191196203656</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-1.617384178139626</v>
+        <v>-1.617384178006098</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>51.00187790428424</v>
+        <v>51.00187792270095</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>9.582401048164582</v>
+        <v>9.58240110446844</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>0.5925048141016146</v>
@@ -5997,7 +5997,7 @@
         <v/>
       </c>
       <c r="D105" s="2" t="n">
-        <v>219.7508490207584</v>
+        <v>219.7508490207583</v>
       </c>
       <c r="E105" s="2" t="n">
         <v>31</v>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>40.42759522567731</v>
+        <v>40.42759490887519</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>16.12340717189815</v>
+        <v>16.12340702784996</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>0.9712822687170788</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>-0.06640604988487921</v>
+        <v>-0.0664060496623365</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6050,7 +6050,7 @@
         <v/>
       </c>
       <c r="D106" s="2" t="n">
-        <v>218.1916297149148</v>
+        <v>218.1916297149147</v>
       </c>
       <c r="E106" s="2" t="n">
         <v>66.8</v>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>40.64570655143384</v>
+        <v>40.64570591105167</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>16.72310016194607</v>
+        <v>16.72310035565432</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.3842965200795153</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>0.0563361940359659</v>
+        <v>0.056336196595196</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>42.39926394793338</v>
+        <v>42.39926393075563</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>17.88937333038178</v>
+        <v>17.88937324759421</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>0.4906624309335515</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.042079592498069</v>
+        <v>0.042079592493617</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6173,7 +6173,7 @@
         <v>41.18486397076366</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>25.17777581015171</v>
+        <v>25.17777598685777</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.1560370124023627</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>0.2439083008681148</v>
+        <v>0.2439083012019183</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>210.5071497297922</v>
+        <v>210.5071497297923</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>68.7</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>52.50052028722487</v>
+        <v>52.50052028919895</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>7.284511759853149</v>
+        <v>7.284511779790938</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.7663444135434601</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>3.511323960267912</v>
+        <v>3.511323960245661</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>49.84962794849375</v>
+        <v>49.84962784452854</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>14.96897802550654</v>
+        <v>14.96897803690279</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.340937166016628</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.1332983693856485</v>
+        <v>0.1332983692521274</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>42.96360611680451</v>
+        <v>42.9636061003958</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>13.65012188801317</v>
+        <v>13.65012190504641</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.3492694072126049</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>-3.072055937577112</v>
+        <v>-3.072055929787922</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>44.6429955097758</v>
+        <v>44.64299542246894</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>11.33901589869094</v>
+        <v>11.33901611770217</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.171532096810977</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>-0.1894128214576416</v>
+        <v>-0.1894128211905856</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>51.35035177071</v>
+        <v>51.35035176281124</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>15.03185935933276</v>
+        <v>15.03185938905215</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.4292346496648372</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>0.590005986673495</v>
+        <v>0.5900059864620837</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>45.09518525138712</v>
+        <v>45.09518515535984</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>19.47250757803604</v>
+        <v>19.47250761671977</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.3841622350083522</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>0.0332903888543798</v>
+        <v>0.0332903889433929</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6527,7 +6527,7 @@
         <v/>
       </c>
       <c r="D115" s="2" t="n">
-        <v>201.3622389803224</v>
+        <v>201.3622389803221</v>
       </c>
       <c r="E115" s="2" t="n">
         <v>58.8</v>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>41.5707361993773</v>
+        <v>41.57073586312946</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>15.21822528847986</v>
+        <v>15.21822538154082</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.8489138037649396</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-0.1784904211411517</v>
+        <v>-0.1784904208518453</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>39.76733161682601</v>
+        <v>39.7673316270852</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>14.19198682046007</v>
+        <v>14.19198682471676</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.6646540163261692</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>-103.6076043101722</v>
+        <v>-103.6076043090593</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>44.64011769358486</v>
+        <v>44.64011697971431</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>17.95638218800901</v>
+        <v>17.95638244072002</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.4594244036317838</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.0701520634526772</v>
+        <v>0.0701520640090348</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6686,7 +6686,7 @@
         <v/>
       </c>
       <c r="D118" s="2" t="n">
-        <v>163.1362691119623</v>
+        <v>163.1362691119624</v>
       </c>
       <c r="E118" s="2" t="n">
         <v>214</v>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>40.6331859742882</v>
+        <v>40.63318601358881</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>23.83361609181967</v>
+        <v>23.83361613542643</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.4603245019449106</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>1.755236778767847</v>
+        <v>1.755236777655147</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>40.19107130303673</v>
+        <v>40.19107121643533</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>18.90451298494492</v>
+        <v>18.9045129195916</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.3759934576631873</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>-1.140880203928835</v>
+        <v>-1.140880203261238</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>40.67576528381733</v>
+        <v>40.67576526452634</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>10.32187124278139</v>
+        <v>10.32187125601145</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.4807071250994642</v>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>35.93313370998274</v>
+        <v>35.9331331900931</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>14.42531088453532</v>
+        <v>14.42531105259587</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.5912643743928939</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.0329445668122498</v>
+        <v>-0.0329445665297319</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>39.42566513308714</v>
+        <v>39.42566507280775</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>16.00938919368576</v>
+        <v>16.00938923272324</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.7665949264223837</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>-0.0026604641302202</v>
+        <v>-0.002660464107969</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>36.12839490395181</v>
+        <v>36.12839461044671</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>18.83398912186306</v>
+        <v>18.83398935270392</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>0.5171171932398859</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>-0.2774329463868292</v>
+        <v>-0.2774329457192123</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>52.40256113611493</v>
+        <v>52.40256183346735</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>6.589316137835839</v>
+        <v>6.589316793723308</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.1717163096355722</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>0.6680866409396138</v>
+        <v>0.6680866333509148</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>45.49448746739471</v>
+        <v>45.4944871939868</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>14.33591616651753</v>
+        <v>14.33591624047454</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.3107575909571903</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>0.9009519548036886</v>
+        <v>0.900951955693848</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7110,7 +7110,7 @@
         <v/>
       </c>
       <c r="D126" s="2" t="n">
-        <v>124.0154397632358</v>
+        <v>124.015439763236</v>
       </c>
       <c r="E126" s="2" t="n">
         <v>57.6</v>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>27.29818946411157</v>
+        <v>27.29819017371364</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>18.97000897750958</v>
+        <v>18.97000894220944</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>1.056226180281053</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-0.2484329955515352</v>
+        <v>-0.2484329956628056</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7163,7 +7163,7 @@
         <v/>
       </c>
       <c r="D127" s="2" t="n">
-        <v>76.11441673857348</v>
+        <v>76.11441673857388</v>
       </c>
       <c r="E127" s="2" t="n">
         <v>40.6</v>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>45.04276454418875</v>
+        <v>45.04276461327216</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>12.73002418027572</v>
+        <v>12.73002418955659</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.3409157264369457</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>0.1591318839263277</v>
+        <v>0.1591318841266165</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>

</xml_diff>